<commit_message>
CS: usa la forza assiale calcolata per candidato nel check di stress
Il driver legacy CS_opt_VNS.m calcolava FZmax con emag() e lo
sovrascriveva con un 35 hardcoded per ogni candidato. Per decisione
dell'utente la forza va definita caso per caso: scan_wp_designs.m ora
passa a eqv_stress_coil_cicc il FZmax calcolato da emag_field_forces
per quel candidato (in MN) e lo salva nella colonna Fz_MN. Rimosso il
parametro F_z_check_MN dal template Excel (38 parametri) e dalla
validazione in read_machine_input.m.

Effetto: S_ver, e quindi S_T_max, non coincidono più con quelli di
CS_opt_VNS.m; il confronto di validazione col legacy va fatto tenendone
conto. Non eseguito in MATLAB in questo ambiente.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019fUkKuwxJNSN93CW6uHDhQ
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/CS/input/WP_CS_input_template.xlsx
+++ b/MADE-2.0/matlab/CS/input/WP_CS_input_template.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1283,25 +1283,25 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Materials &amp; allowables</t>
+          <t>Geometric consistency checks</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>F_z_check_MN</t>
+          <t>SC_w_min</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>35</v>
+        <v>0.005</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Axial force used in the final stress check. OPEN QUESTION: the legacy driver (CS_opt_VNS.m) computed FZmax from EMAG_FIELD_FORCES and then immediately overwrote it with this fixed value - carried over unchanged, see manuale CS 'decisioni aperte'.</t>
+          <t>Minimum admissible SC cable width</t>
         </is>
       </c>
     </row>
@@ -1313,20 +1313,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SC_w_min</t>
+          <t>r_cable_min</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.005</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Minimum admissible SC cable width</t>
+          <t>Minimum admissible cable aspect ratio Cond_h/Cond_w</t>
         </is>
       </c>
     </row>
@@ -1338,11 +1338,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>r_cable_min</t>
+          <t>r_cable_max</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Minimum admissible cable aspect ratio Cond_h/Cond_w</t>
+          <t>Maximum admissible cable aspect ratio Cond_h/Cond_w</t>
         </is>
       </c>
     </row>
@@ -1363,20 +1363,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>r_cable_max</t>
+          <t>JT_min_check</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2.5</v>
+        <v>0.001</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Maximum admissible cable aspect ratio Cond_h/Cond_w</t>
+          <t>Minimum admissible jacket thickness (post-sizing check)</t>
         </is>
       </c>
     </row>
@@ -1388,11 +1388,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>JT_min_check</t>
+          <t>Ri_min</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.001</v>
+        <v>0.3</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1400,31 +1400,6 @@
         </is>
       </c>
       <c r="E39" t="inlineStr">
-        <is>
-          <t>Minimum admissible jacket thickness (post-sizing check)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Geometric consistency checks</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Ri_min</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
         <is>
           <t>Minimum admissible winding-pack inner radius</t>
         </is>
@@ -1508,7 +1483,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>This is a direct port of CS_opt_VNS.m (2026-09-29). See the 'Manuale CS' artifact for the full legacy-file</t>
+          <t>This is a direct port of CS_opt_VNS.m (2026-09-29, updated 2026-10-01). See the 'Manuale CS' artifact for the full legacy-file</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1497,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>(notably F_z_check_MN and the Ic_sst33 argument order, see the corresponding cell/function comments).</t>
+          <t>(notably the Ic_sst33 argument order in the HTS branch, see the corresponding function comment).</t>
         </is>
       </c>
     </row>

</xml_diff>